<commit_message>
Project CopyTable is saved.
</commit_message>
<xml_diff>
--- a/CopyTable/CopyTable.xlsx
+++ b/CopyTable/CopyTable.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10726"/>
   <workbookPr defaultThemeVersion="202300"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <mc:AlternateContent>
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ekosolapova/Downloads/"/>
     </mc:Choice>
@@ -17,7 +17,7 @@
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+    <ext uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="10">
   <si>
     <r>
       <rPr>
@@ -102,11 +102,15 @@
   <si>
     <t>&gt; 10</t>
   </si>
+  <si>
+    <t>SimpleRules Double CreditPortfolioQualityScore2 (Double creditPortfolioQuality)</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="0"/>
   <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
@@ -323,7 +327,7 @@
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellStyleXfs>
   <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -691,10 +695,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A03E2933-7A64-6C43-9288-7F9C64316259}">
-  <dimension ref="C6:D13"/>
+  <dimension ref="B6:D22"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="4" max="4" width="49.83203125" customWidth="1"/>
+    <col min="4" max="4" customWidth="true" width="49.83203125"/>
   </cols>
   <sheetData>
     <row r="6" spans="3:4" ht="20" thickBot="1" x14ac:dyDescent="0.35">
@@ -759,9 +763,72 @@
         <v>0</v>
       </c>
     </row>
+    <row r="15">
+      <c r="B15" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="C15" s="0"/>
+    </row>
+    <row r="16">
+      <c r="B16" t="s" s="0">
+        <v>1</v>
+      </c>
+      <c r="C16" t="s" s="0">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="C17" t="n" s="0">
+        <v>1.0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C18" t="n" s="0">
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" t="s" s="0">
+        <v>5</v>
+      </c>
+      <c r="C19" t="n" s="0">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" t="s" s="0">
+        <v>6</v>
+      </c>
+      <c r="C20" t="n" s="0">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="C21" t="n" s="0">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" t="s" s="0">
+        <v>8</v>
+      </c>
+      <c r="C22" t="n" s="0">
+        <v>0.0</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="2">
     <mergeCell ref="C6:D6"/>
+    <mergeCell ref="B15:C15"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>